<commit_message>
Flatten JR outputs and rename map intermediates for clarity.
Drop legacy result/visualization folders and matched_entities_log; use cross_group_map.xlsx and within_group.xlsx; remove unused __init__.py files.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/output/jr_database/RA_workpack.xlsx
+++ b/output/jr_database/RA_workpack.xlsx
@@ -483,12 +483,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>目的</t>
+          <t>Purpose</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>一本檔處理三件事：名字 resolve、Sheet2 互惠缺漏、把 Keerthana/llm 補進 ICMID Sheet2/3。</t>
+          <t>One workbook for three tasks: resolve names, fix Sheet2 reciprocity gaps, and import Keerthana/llm pairs into ICMID Sheet2/3.</t>
         </is>
       </c>
     </row>
@@ -499,36 +499,36 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>總原則</t>
+          <t>Principle</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>先 resolve 名字，再判斷漏打／互惠。沒 resolve 的拼寫不要當漏打。</t>
+          <t>Resolve names first, then judge missing / one-sided links. Unresolved spellings are not missing reverse links.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Resolve 順序</t>
+          <t>Resolve order</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>ethnic_entity_index → registry aliases → GIS exact（murdock → greg → geopr）。</t>
+          <t>ethnic_entity_index → registry aliases → GIS exact (murdock → greg → geopr).</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>合法 polygon_source</t>
+          <t>Allowed polygon_source</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>只填 murdock / greg / geopr（不要填 Joshua Project）。</t>
+          <t>Only murdock / greg / geopr (do not use Joshua Project).</t>
         </is>
       </c>
     </row>
@@ -539,48 +539,48 @@
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>STEP 1 — 對名字（必做）</t>
+          <t>STEP 1 — Resolve names (required)</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>開 sheet：1_unmatched_entities</t>
+          <t>Open sheet: 1_unmatched_entities</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>做什麼</t>
+          <t>What to do</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>entity 還對不上 homeland。填 polygon_source、polygon_id；可選 display_name / resolve_source / aliases。</t>
+          <t>Entities still without a homeland. Fill polygon_source, polygon_id; optional display_name / resolve_source / aliases.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>範例</t>
+          <t>Example</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Maasai → murdock / MASAI（雙 a 拼寫要手動對到 Murdock MASAI）。</t>
+          <t>Maasai → murdock / MASAI (double-a spelling must be mapped to Murdock MASAI).</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>做完後</t>
+          <t>After filling</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>存檔，執行：uv run python -B code/jr_database/build_cross_group.py --apply-unmatched</t>
+          <t>Save, then run: uv run python -B code/jr_database/build_cross_group.py --apply-unmatched</t>
         </is>
       </c>
     </row>
@@ -591,36 +591,36 @@
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>STEP 1b — Sheet2 裡未 resolve 的 partner</t>
+          <t>STEP 1b — Unresolved Sheet2 partners</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>開 sheet：1b_unresolved_partners</t>
+          <t>Open sheet: 1b_unresolved_partners</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>做什麼</t>
+          <t>What to do</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Sheet2 Joking link 裡的拼寫對不上（如 Zaramu、Kami）。同樣填進 1_unmatched_entities 或 index alias，再 --apply-unmatched。</t>
+          <t>Spellings in Sheet2 Joking link that do not resolve (e.g. Zaramu, Kami). Add them to 1_unmatched_entities or an index alias, then --apply-unmatched.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>注意</t>
+          <t>Note</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>這些不算「漏打反向」；先 alias 再重跑 workpack 看 2_missing_reverse。</t>
+          <t>These are not missing reverse links; alias first, then re-export the workpack and check 2_missing_reverse.</t>
         </is>
       </c>
     </row>
@@ -631,36 +631,36 @@
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>STEP 2 — Sheet2 單邊缺反向</t>
+          <t>STEP 2 — Sheet2 missing reverse</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>開 sheet：2_missing_reverse</t>
+          <t>Open sheet: 2_missing_reverse</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>做什麼</t>
+          <t>What to do</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>has_link 已寫 partner；missing_on 那列沒寫回來。在 ICMID- Africa.xlsx Sheet2 補 should_add，或從 has_link 刪掉並註記。</t>
+          <t>has_link already lists the partner; missing_on does not list back. Add should_add on ICMID- Africa.xlsx Sheet2, or remove from has_link and note why.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>若有 unresolved spellings</t>
+          <t>If unresolved spellings remain</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>先做 STEP 1b，再重跑 export，避免誤判。</t>
+          <t>Finish STEP 1b first, then re-export to avoid false positives.</t>
         </is>
       </c>
     </row>
@@ -671,36 +671,36 @@
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>STEP 2b — partner 無 Sheet2 列</t>
+          <t>STEP 2b — Partner has no Sheet2 row</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>開 sheet：2b_partner_not_in_sheet2</t>
+          <t>Open sheet: 2b_partner_not_in_sheet2</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>意思</t>
+          <t>Meaning</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>A 寫了 B，B 有 resolve，但 Sheet2 沒有 B 那列（常是 GREG/GeoEPR）。無法在 Sheet2 補反向。</t>
+          <t>A lists B, B resolves, but Sheet2 has no row for B (often GREG/GeoEPR). Cannot add a Sheet2 reverse link.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>怎麼處理</t>
+          <t>How to handle</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>接受為額外族群；或確認是否應新建 Murdock 列；不要硬當 missing_reverse。</t>
+          <t>Accept as an extra group, or confirm whether a Murdock row should be created; do not treat as missing_reverse.</t>
         </is>
       </c>
     </row>
@@ -711,36 +711,36 @@
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>STEP 3 — 把其他來源補進 ICMID</t>
+          <t>STEP 3 — Import other sources into ICMID</t>
         </is>
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>開 sheet：3_to_sheet2 與 3_to_sheet3</t>
+          <t>Open sheets: 3_to_sheet2 and 3_to_sheet3</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>規則（老師）</t>
+          <t>Rule (advisor)</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>pair 至少一邊是 murdock → Sheet2；兩邊都不是 → Sheet3。</t>
+          <t>If at least one endpoint is murdock → Sheet2; if neither is → Sheet3.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>來源</t>
+          <t>Sources</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>keerthana_analysis + llm_ehraf（不含 keerthana og）。</t>
+          <t>keerthana_analysis + llm_ehraf (not keerthana og).</t>
         </is>
       </c>
     </row>
@@ -752,7 +752,7 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>status=add_partner… → 在既有 Sheet2 列的 Joking link 加上 partner_to_add；create_new… → 先新建 Ethnic Group 列。</t>
+          <t>status=add_partner… → append partner_to_add on the existing Sheet2 Joking link; create_new… → create an Ethnic Group row first.</t>
         </is>
       </c>
     </row>
@@ -764,7 +764,7 @@
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>兩邊都不是 murdock，候補進 Sheet3。先丟掉過泛名稱（villagers、Europeans、males…）。</t>
+          <t>Neither side is murdock; candidate for Sheet3. Drop overly generic names (villagers, Europeans, males, …) first.</t>
         </is>
       </c>
     </row>
@@ -776,7 +776,7 @@
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>已在 Sheet2，可略過。</t>
+          <t>Already on Sheet2; skip.</t>
         </is>
       </c>
     </row>
@@ -787,19 +787,19 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>建議順序</t>
+          <t>Suggested order</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>1 → 1b → apply-unmatched → 重跑本 workpack → 2 → 2b → 3。</t>
+          <t>1 → 1b → apply-unmatched → re-export this workpack → 2 → 2b → 3.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>重跑指令</t>
+          <t>Re-run commands</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
@@ -811,24 +811,24 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>主檔</t>
+          <t>Primary coding file</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>data/sources/ICMID- Africa.xlsx（Sheet2 主編碼；Sheet3 暫存）。</t>
+          <t>data/sources/ICMID- Africa.xlsx (Sheet2 main coding; Sheet3 holding).</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>長期對照表</t>
+          <t>Long-term lookup</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>data/lookup/ethnic_entity_index.xlsx（apply 後寫入；勿只改 workpack 不 apply）。</t>
+          <t>data/lookup/ethnic_entity_index.xlsx (written on apply; do not edit only the workpack).</t>
         </is>
       </c>
     </row>

</xml_diff>